<commit_message>
Photo framing, owner name, custom categories, and AI description help
Every maker photo frame is 4:3 (work photos square) and people frame their
photo in that exact shape before upload, with a whole image option for logos.
Minimum sizes drop to 800 x 600 and 800 x 800. Listings get an owner name,
makers can type their own category for owner approval, and a Workers AI
helper suggests a polished short description (free tier, 15 per maker a day).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hXCRRqaTS4Zyqv7movrZd
</commit_message>
<xml_diff>
--- a/client/public/downloads/Vendor-Bulk-Import-Template.xlsx
+++ b/client/public/downloads/Vendor-Bulk-Import-Template.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P250"/>
+  <dimension ref="A1:Q250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,7 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -570,6 +571,11 @@
           <t>login_email</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>owner_name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -638,6 +644,11 @@
           <t>maker@example.com</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Jane Maker</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -4876,7 +4887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -4949,44 +4960,51 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>8. Optional: owner_name is the owner's full name, shown on the profile as "Meet" and their name.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Security and privacy</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Do not include passwords, payment information, government IDs, or private notes in this file.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="n"/>
-    </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Allowed social domains</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Instagram: instagram.com  |  Facebook: facebook.com or fb.com  |  TikTok: tiktok.com</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="n"/>
+    <row r="19">
+      <c r="A19" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Optional links with @handles, one step maker invites, compatible import template
Website and social links are optional for makers and applicants, and handles or
bare domains are saved as full links. Approve and invite now starts the maker's
listing from their application, and Published vendors rows get Invite maker
and Welcome email. The import reads any template version by column name, skips
unknown columns, and the template instructions are updated (version 3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hXCRRqaTS4Zyqv7movrZd
</commit_message>
<xml_diff>
--- a/client/public/downloads/Vendor-Bulk-Import-Template.xlsx
+++ b/client/public/downloads/Vendor-Bulk-Import-Template.xlsx
@@ -610,12 +610,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://example.com</t>
+          <t>examplemaker.com</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/examplemaker</t>
+          <t>@examplemaker</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -4896,112 +4896,120 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>The Cannery Marketplace — One-Time Vendor Import</t>
+          <t>The Cannery Marketplace: Vendor Import (template version 3, October 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>How to use this file</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>1. Keep the header row unchanged. Fields marked with * are required.</t>
+          <t>1. Add one vendor per row. Delete the example row before importing real vendors.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2. Add one vendor per row. Delete the example row before importing real vendors.</t>
+          <t>2. Required for every row: name, category, short_bio (at least 20 characters), and an email (contact_email, or login_email if they are the same).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>3. Social links must point to the matching service (Instagram, Facebook, or TikTok).</t>
+          <t>3. Everything else is optional, including website and social media.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>4. Separate multiple gallery image URLs with a vertical bar: URL 1 | URL 2. Maximum five gallery images.</t>
+          <t>4. Website: a full link or just the address, like examplemaker.com.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>5. Save as .xlsx, upload in Admin &gt; Vendor import, review all errors, then confirm the import.</t>
+          <t>5. Instagram, Facebook, TikTok: type the @handle (like @examplemaker) or paste the full link.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>6. Imported vendors are approved by the administrator and can appear publicly when Active is Yes.</t>
+          <t>6. login_email: the email the maker signs in with to edit their listing. It is added to Maker access automatically. One email can be used on several rows.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>7. Optional: login_email is the email the maker signs in with to edit their listing. It is added to Maker access automatically. One email can be used on several rows.</t>
+          <t>7. owner_name: the owner's full name, shown on the profile as "Meet" and their name.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>8. Optional: owner_name is the owner's full name, shown on the profile as "Meet" and their name.</t>
+          <t>8. Gallery images: separate several links with a vertical bar (|). Maximum five.</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>9. featured and active: Yes or No. display_order: a number; lower numbers show first.</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>10. Save as .xlsx, upload in the owner dashboard under Vendor import, fix any problems shown, then confirm.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Works with any version</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Columns can be in any order and any letter case, with or without the * marks. Older versions of this template still import. Columns the site does not recognize are listed and skipped, so adding your own notes column is safe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Security and privacy</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Do not include passwords, payment information, government IDs, or private notes in this file.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="n"/>
-    </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Allowed social domains</t>
-        </is>
-      </c>
+      <c r="A17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Instagram: instagram.com  |  Facebook: facebook.com or fb.com  |  TikTok: tiktok.com</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>

</xml_diff>

<commit_message>
Use Maker's full name and Business name consistently
Renames Owner's full name to Maker's full name across the listing editor,
maker portal, review queue, messages, and AI helper, and Business or maker name
to Business name. The import column becomes maker_full_name; owner_name still
imports.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hXCRRqaTS4Zyqv7movrZd
</commit_message>
<xml_diff>
--- a/client/public/downloads/Vendor-Bulk-Import-Template.xlsx
+++ b/client/public/downloads/Vendor-Bulk-Import-Template.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>owner_name</t>
+          <t>maker_full_name</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2. Required for every row: name, category, short_bio (at least 20 characters), and an email (contact_email, or login_email if they are the same).</t>
+          <t>2. Required for every row: name (the business name), category, short_bio (at least 20 characters), and an email (contact_email, or login_email if they are the same).</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>7. owner_name: the owner's full name, shown on the profile as "Meet" and their name.</t>
+          <t>7. maker_full_name: the maker's full name (the person behind the work), shown on the profile as "Meet" and their name. Older files that use owner_name still work.</t>
         </is>
       </c>
     </row>

</xml_diff>